<commit_message>
refactor: implement all 14 changes from problem statement
Agent-Logs-Url: https://github.com/SaeedR1987/public_health_resources/sessions/9d047d00-cf31-4b0e-a6f4-94c246fbf3ab

Co-authored-by: SaeedR1987 <17695865+SaeedR1987@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/inst/resources/tool_household_iphra_v2.xlsx
+++ b/inst/resources/tool_household_iphra_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection lockStructure="1" workbookAlgorithmName="SHA-512" workbookHashValue="h2fYSiQvhiNGkrtUsLkSn45g315KWDSA25bD4j3ORM5bRlKWMnBDtzvS6AbBSYAj6ag3ODyY1mEUTQPcGFJ0Tg==" workbookSaltValue="IfpCe47h0g637JARLrp1Sg==" workbookSpinCount="100000"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_Me" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Read_Me" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'survey'!$B$1:$R$337</definedName>
@@ -995,42 +995,42 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>label::French (fr)</t>
+          <t>label::French</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>hint::French (fr)</t>
+          <t>hint::French</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>label::Arabic (ar)</t>
+          <t>label::Arabic</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>hint::Arabic (ar)</t>
+          <t>hint::Arabic</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>label::Spanish (sp)</t>
+          <t>label::Spanish</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>hint::Spanish (sp)</t>
+          <t>hint::Spanish</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>label::English (en)</t>
+          <t>label::English</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>hint::English (en)</t>
+          <t>hint::English</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
@@ -15590,22 +15590,22 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>label::French (fr)</t>
+          <t>label::French</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>label::Arabic (ar)</t>
+          <t>label::Arabic</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>label::Spanish (sp)</t>
+          <t>label::Spanish</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>label::English (en)</t>
+          <t>label::English</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">

</xml_diff>